<commit_message>
Fixed three bugs in the mass_update_templates.py script: - The script was not working correctly when there were no replacements to make - The script was not working correctly when there were no text nodes to replace - The script was not working correctly when there were no matches to replace
</commit_message>
<xml_diff>
--- a/Testing_Files/ClioCustomField_TestValidation.xlsx
+++ b/Testing_Files/ClioCustomField_TestValidation.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/Testing_Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="939" documentId="8_{3120D6FD-25C6-47F0-8A39-89B25F99CA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6EEB7DC-2F34-456E-925D-DDBE26C93942}"/>
+  <xr:revisionPtr revIDLastSave="988" documentId="8_{3120D6FD-25C6-47F0-8A39-89B25F99CA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94A7E552-2C4D-4223-8F0A-6C283B855932}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DF2C5E22-660C-4BCB-A765-9F1A84EF46AA}"/>
+    <workbookView xWindow="3165" yWindow="1365" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{DF2C5E22-660C-4BCB-A765-9F1A84EF46AA}"/>
   </bookViews>
   <sheets>
     <sheet name="FunctionalTestScenarios" sheetId="1" r:id="rId1"/>
-    <sheet name="EdgeCaseTestingScenarios" sheetId="3" r:id="rId2"/>
-    <sheet name="Templates" sheetId="2" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId2"/>
+    <sheet name="EdgeCaseTestingScenarios" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FunctionalTestScenarios!$A$1:$F$5</definedName>
-    <definedName name="_Hlk108346204" localSheetId="1">EdgeCaseTestingScenarios!$D$12</definedName>
+    <definedName name="_Hlk108346204" localSheetId="2">EdgeCaseTestingScenarios!$D$12</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="142">
   <si>
     <t>TempCode</t>
   </si>
@@ -53,30 +53,6 @@
     <t>NewFieldCodes</t>
   </si>
   <si>
-    <t xml:space="preserve">TESTING DOC </t>
-  </si>
-  <si>
-    <t>TESTING DOC NAME</t>
-  </si>
-  <si>
-    <t>Template 1</t>
-  </si>
-  <si>
-    <t>Meet and Confer Letter re Plaintiff's MILs 1-21 (Single Pltf)</t>
-  </si>
-  <si>
-    <t>Template 2</t>
-  </si>
-  <si>
-    <t>Demand for Exchange of Expert (Singular Plaintiff)</t>
-  </si>
-  <si>
-    <t>Template 3</t>
-  </si>
-  <si>
-    <t>Decl ISO Expert Designation of Plaintiff's Experts (Singular Plaintiff)</t>
-  </si>
-  <si>
     <t>Outcome - Successful?</t>
   </si>
   <si>
@@ -746,6 +722,93 @@
   </si>
   <si>
     <t>&lt;&lt; User.Name_UPDATED_030526 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>Old_Value</t>
+  </si>
+  <si>
+    <t>New_Value</t>
+  </si>
+  <si>
+    <t>&lt;&lt; date.verbose &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; date.verbose_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.casenumber &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.casenumber_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.county &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.county_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DefendantsNameShort &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DefendantsNameShort_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleYear_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CaseNameShort &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CaseNameShort_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CourtStreetAddress &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CourtStreetAddress_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; TestCustomField.Test &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;  TestCustomField.Test_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>CMS AB</t>
+  </si>
+  <si>
+    <t>CMS NonAB</t>
+  </si>
+  <si>
+    <t>NOD DLR 1</t>
+  </si>
+  <si>
+    <t>NOD DLR 2</t>
+  </si>
+  <si>
+    <t>SUBP No. 2</t>
+  </si>
+  <si>
+    <t>SUBP No. 3</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>TextBox</t>
+  </si>
+  <si>
+    <t>Shape</t>
+  </si>
+  <si>
+    <t>Body</t>
+  </si>
+  <si>
+    <t>Footers</t>
+  </si>
+  <si>
+    <t>Headers</t>
   </si>
 </sst>
 </file>
@@ -755,7 +818,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="."/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -815,8 +878,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -838,18 +909,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -901,8 +960,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="24">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -1205,11 +1270,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1219,12 +1308,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1256,7 +1339,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1301,60 +1384,60 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="10" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="10" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="10" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1366,16 +1449,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1393,7 +1476,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1414,54 +1497,55 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1483,14 +1567,40 @@
       </fill>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1511,8 +1621,20 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3E649AE1-97E4-451E-BF3B-1DE7553D5891}" name="Table1" displayName="Table1" ref="A1:G9" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:G9" xr:uid="{3E649AE1-97E4-451E-BF3B-1DE7553D5891}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{C2E1002A-19BA-4B0C-BF86-9D2D029463A4}" name="Old_Value" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{D3150A6E-D425-4799-B9BD-D73C5FB3C4D4}" name="CMS AB"/>
+    <tableColumn id="4" xr3:uid="{9236D882-AF3F-44E4-A0B2-3B49D3143B7B}" name="CMS NonAB"/>
+    <tableColumn id="5" xr3:uid="{4749057A-4E6C-49C5-9C15-3BDC30DC7313}" name="NOD DLR 1"/>
+    <tableColumn id="6" xr3:uid="{7DF7FEBF-1019-4BA4-8A80-571819C75EC3}" name="NOD DLR 2"/>
+    <tableColumn id="7" xr3:uid="{4AD0BB5B-A5CC-4D34-9DF1-727641D2B3F2}" name="SUBP No. 2"/>
+    <tableColumn id="8" xr3:uid="{3BECB5C8-169B-46F9-9419-BE76075774DB}" name="SUBP No. 3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1844,200 +1966,200 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="12" t="s">
+      <c r="B1" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="93" t="s">
-        <v>104</v>
-      </c>
-      <c r="F1" s="22" t="s">
-        <v>11</v>
+      <c r="E1" s="86" t="s">
+        <v>96</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="16"/>
-      <c r="B2" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="C2" s="90" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="90" t="s">
-        <v>106</v>
-      </c>
-      <c r="E2" s="94">
+      <c r="A2" s="12"/>
+      <c r="B2" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="E2" s="12">
         <v>2</v>
       </c>
-      <c r="F2" s="19"/>
+      <c r="F2" s="15"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
-      <c r="B3" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="C3" s="90" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>108</v>
-      </c>
-      <c r="E3" s="94">
+      <c r="A3" s="12"/>
+      <c r="B3" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="E3" s="12">
         <v>1</v>
       </c>
-      <c r="F3" s="19"/>
+      <c r="F3" s="15"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
-      <c r="B4" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="C4" s="91" t="s">
-        <v>109</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="E4" s="94">
+      <c r="A4" s="12"/>
+      <c r="B4" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E4" s="12">
         <v>3</v>
       </c>
-      <c r="F4" s="19"/>
+      <c r="F4" s="15"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
-      <c r="B5" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="C5" s="90" t="s">
-        <v>109</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="E5" s="95">
+      <c r="B5" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E5" s="1">
         <v>3</v>
       </c>
-      <c r="F5" s="9"/>
+      <c r="F5" s="5"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
-      <c r="B6" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="C6" s="92" t="s">
-        <v>112</v>
-      </c>
-      <c r="D6" s="92" t="s">
-        <v>113</v>
-      </c>
-      <c r="E6" s="98">
+      <c r="B6" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="E6" s="89">
         <v>1</v>
       </c>
-      <c r="F6" s="9"/>
+      <c r="F6" s="5"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
-      <c r="B7" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="C7" s="91" t="s">
-        <v>114</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="E7" s="95">
+      <c r="B7" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="1">
         <v>1</v>
       </c>
-      <c r="F7" s="9"/>
+      <c r="F7" s="5"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
-      <c r="B8" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="C8" s="90" t="s">
-        <v>109</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="E8" s="95">
+      <c r="B8" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E8" s="1">
         <v>3</v>
       </c>
-      <c r="F8" s="9"/>
+      <c r="F8" s="5"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
-      <c r="B9" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="C9" s="90" t="s">
-        <v>117</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="E9" s="95">
+      <c r="B9" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" s="1">
         <v>1</v>
       </c>
-      <c r="F9" s="9"/>
+      <c r="F9" s="5"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="C10" s="91" t="s">
-        <v>119</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="E10" s="96">
+      <c r="B10" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E10" s="87">
         <v>2</v>
       </c>
-      <c r="F10" s="13"/>
+      <c r="F10" s="9"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
       <c r="D11" s="2"/>
-      <c r="E11" s="96"/>
-      <c r="F11" s="13"/>
+      <c r="E11" s="87"/>
+      <c r="F11" s="9"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="96"/>
-      <c r="F12" s="13"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="87"/>
+      <c r="F12" s="9"/>
     </row>
     <row r="13" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
       <c r="D13" s="4"/>
-      <c r="E13" s="97"/>
-      <c r="F13" s="14"/>
+      <c r="E13" s="88"/>
+      <c r="F13" s="10"/>
     </row>
     <row r="21" spans="4:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="D21" s="15"/>
+      <c r="D21" s="11"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F5" xr:uid="{BDCEFEA6-5597-44CB-97F0-1FAC3A383FDA}"/>
   <conditionalFormatting sqref="D3">
-    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
@@ -2047,568 +2169,832 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{622E4ABB-CB79-43BB-AA1D-E9B06737D8D9}">
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="56.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="90" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" s="90" t="s">
+        <v>130</v>
+      </c>
+      <c r="C1" s="90" t="s">
+        <v>131</v>
+      </c>
+      <c r="D1" s="90" t="s">
+        <v>132</v>
+      </c>
+      <c r="E1" s="90" t="s">
+        <v>133</v>
+      </c>
+      <c r="F1" s="90" t="s">
+        <v>134</v>
+      </c>
+      <c r="G1" s="90" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="97" t="s">
+        <v>136</v>
+      </c>
+      <c r="B11" s="55"/>
+      <c r="C11" s="55"/>
+      <c r="D11" s="55"/>
+      <c r="E11" s="55"/>
+      <c r="F11" s="55"/>
+      <c r="G11" s="55"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+    </row>
+    <row r="16" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="95" t="s">
+        <v>114</v>
+      </c>
+      <c r="B18" s="95" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" s="95" t="s">
+        <v>131</v>
+      </c>
+      <c r="D18" s="95" t="s">
+        <v>132</v>
+      </c>
+      <c r="E18" s="95" t="s">
+        <v>133</v>
+      </c>
+      <c r="F18" s="95" t="s">
+        <v>134</v>
+      </c>
+      <c r="G18" s="96" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="93" t="s">
+        <v>116</v>
+      </c>
+      <c r="B19" s="93"/>
+      <c r="C19" s="93"/>
+      <c r="D19" s="93"/>
+      <c r="E19" s="93"/>
+      <c r="F19" s="93"/>
+      <c r="G19" s="91"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="94" t="s">
+        <v>118</v>
+      </c>
+      <c r="B20" s="94"/>
+      <c r="C20" s="94"/>
+      <c r="D20" s="94"/>
+      <c r="E20" s="94"/>
+      <c r="F20" s="94"/>
+      <c r="G20" s="92"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="93" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" s="93"/>
+      <c r="C21" s="93"/>
+      <c r="D21" s="93"/>
+      <c r="E21" s="93"/>
+      <c r="F21" s="93"/>
+      <c r="G21" s="91"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B22" s="94"/>
+      <c r="C22" s="94"/>
+      <c r="D22" s="94"/>
+      <c r="E22" s="94"/>
+      <c r="F22" s="94"/>
+      <c r="G22" s="92"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="93" t="s">
+        <v>123</v>
+      </c>
+      <c r="B23" s="93"/>
+      <c r="C23" s="93"/>
+      <c r="D23" s="93"/>
+      <c r="E23" s="93"/>
+      <c r="F23" s="93"/>
+      <c r="G23" s="91"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="94" t="s">
+        <v>125</v>
+      </c>
+      <c r="B24" s="94"/>
+      <c r="C24" s="94"/>
+      <c r="D24" s="94"/>
+      <c r="E24" s="94"/>
+      <c r="F24" s="94"/>
+      <c r="G24" s="92"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="93" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="93"/>
+      <c r="C25" s="93"/>
+      <c r="D25" s="93"/>
+      <c r="E25" s="93"/>
+      <c r="F25" s="93"/>
+      <c r="G25" s="91"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="94" t="s">
+        <v>129</v>
+      </c>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="94"/>
+      <c r="F26" s="94"/>
+      <c r="G26" s="92"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F86F2E04-EE71-4EEA-BC46-ACCE4253F69D}">
   <dimension ref="A1:H39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="82.85546875" customWidth="1"/>
-    <col min="3" max="3" width="58.85546875" style="29" customWidth="1"/>
-    <col min="4" max="4" width="53.42578125" style="29" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="74.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.85546875" style="25" customWidth="1"/>
+    <col min="4" max="4" width="53.42578125" style="25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="74.140625" style="25" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="48.5703125" customWidth="1"/>
     <col min="7" max="7" width="51.7109375" customWidth="1"/>
     <col min="8" max="8" width="94.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="29" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45"/>
-      <c r="B1" s="73" t="s">
+    <row r="1" spans="1:8" s="25" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="41"/>
+      <c r="B1" s="69" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="70" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="70" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="70" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="70" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" s="70" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="70" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="45"/>
+      <c r="B2" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="40"/>
+    </row>
+    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="46"/>
+      <c r="B3" s="71" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="72" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="80" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="73" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="50"/>
+      <c r="G3" s="74" t="s">
+        <v>78</v>
+      </c>
+      <c r="H3" s="74"/>
+    </row>
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="46"/>
+      <c r="B4" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="61" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="68" t="s">
+        <v>57</v>
+      </c>
+      <c r="F4" s="51"/>
+      <c r="G4" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="H4" s="19"/>
+    </row>
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="46"/>
+      <c r="B5" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="61" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="81" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="67" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="51"/>
+      <c r="G5" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="H5" s="19"/>
+    </row>
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="46">
+        <v>1</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="61" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="68" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="54" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="H6" s="19"/>
+    </row>
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="46"/>
+      <c r="B7" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="61" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="81" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="67" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="51"/>
+      <c r="G7" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="H7" s="19"/>
+    </row>
+    <row r="8" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="46"/>
+      <c r="B8" s="78" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="77" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="75" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="79" t="s">
+        <v>61</v>
+      </c>
+      <c r="F8" s="52"/>
+      <c r="G8" s="76" t="s">
+        <v>78</v>
+      </c>
+      <c r="H8" s="76"/>
+    </row>
+    <row r="9" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="46"/>
+      <c r="B9" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="61" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="67" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" s="67" t="s">
+        <v>87</v>
+      </c>
+      <c r="F9" s="52"/>
+      <c r="G9" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="H9" s="19"/>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="47"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="75"/>
+      <c r="D10" s="75"/>
+      <c r="E10" s="75"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+    </row>
+    <row r="11" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="45"/>
+      <c r="B11" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="60"/>
+      <c r="D11" s="82" t="s">
+        <v>79</v>
+      </c>
+      <c r="E11" s="82" t="s">
+        <v>80</v>
+      </c>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="40"/>
+    </row>
+    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="46"/>
+      <c r="B12" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="67" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" s="67" t="s">
+        <v>81</v>
+      </c>
+      <c r="F12" s="53"/>
+      <c r="G12" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="H12" s="19"/>
+    </row>
+    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="46"/>
+      <c r="B13" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="68" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" s="68" t="s">
+        <v>82</v>
+      </c>
+      <c r="F13" s="51"/>
+      <c r="G13" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="H13" s="19"/>
+    </row>
+    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="46"/>
+      <c r="B14" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="67" t="s">
+        <v>74</v>
+      </c>
+      <c r="E14" s="67" t="s">
+        <v>83</v>
+      </c>
+      <c r="F14" s="51"/>
+      <c r="G14" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="H14" s="19"/>
+    </row>
+    <row r="15" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="46">
+        <v>2</v>
+      </c>
+      <c r="B15" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="74" t="s">
+      <c r="C15" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="68" t="s">
+        <v>76</v>
+      </c>
+      <c r="E15" s="68" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" s="54" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="H15" s="19"/>
+    </row>
+    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="46"/>
+      <c r="B16" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" s="67" t="s">
+        <v>54</v>
+      </c>
+      <c r="E16" s="67" t="s">
+        <v>85</v>
+      </c>
+      <c r="F16" s="51"/>
+      <c r="G16" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="H16" s="19"/>
+    </row>
+    <row r="17" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="46"/>
+      <c r="B17" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="68" t="s">
+        <v>77</v>
+      </c>
+      <c r="E17" s="68" t="s">
+        <v>86</v>
+      </c>
+      <c r="F17" s="51"/>
+      <c r="G17" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="H17" s="19"/>
+    </row>
+    <row r="18" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="47"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="62"/>
+      <c r="D18" s="62"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="55"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+    </row>
+    <row r="19" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="45"/>
+      <c r="B19" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="74" t="s">
-        <v>76</v>
-      </c>
-      <c r="E1" s="74" t="s">
-        <v>77</v>
-      </c>
-      <c r="F1" s="74" t="s">
+      <c r="C19" s="60"/>
+      <c r="D19" s="60"/>
+      <c r="E19" s="60"/>
+      <c r="F19" s="49"/>
+      <c r="G19" s="39"/>
+      <c r="H19" s="40"/>
+    </row>
+    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="46"/>
+      <c r="B20" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="61" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" s="67" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="67" t="s">
+        <v>89</v>
+      </c>
+      <c r="F20" s="57"/>
+      <c r="G20" s="56" t="s">
+        <v>78</v>
+      </c>
+      <c r="H20" s="14"/>
+    </row>
+    <row r="21" spans="1:8" s="25" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A21" s="42">
+        <v>3</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" s="59" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="54" t="s">
+        <v>53</v>
+      </c>
+      <c r="G21" s="84" t="s">
+        <v>78</v>
+      </c>
+      <c r="H21" s="1"/>
+    </row>
+    <row r="22" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="46"/>
+      <c r="B22" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="59" t="s">
+        <v>38</v>
+      </c>
+      <c r="D22" s="83" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="83" t="s">
+        <v>91</v>
+      </c>
+      <c r="F22" s="58"/>
+      <c r="G22" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="H22" s="2"/>
+    </row>
+    <row r="23" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="47"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="63"/>
+      <c r="D23" s="63"/>
+      <c r="E23" s="63"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="30"/>
+    </row>
+    <row r="24" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="45"/>
+      <c r="B24" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" s="60"/>
+      <c r="D24" s="60"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="39"/>
+      <c r="G24" s="39"/>
+      <c r="H24" s="40"/>
+    </row>
+    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="46"/>
+      <c r="B25" s="33" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G1" s="74" t="s">
+      <c r="F25" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="G25" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="H25" s="14"/>
+    </row>
+    <row r="26" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A26" s="46">
+        <v>4</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="H1" s="74" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="49"/>
-      <c r="B2" s="42" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="44"/>
-    </row>
-    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="50"/>
-      <c r="B3" s="75" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" s="76" t="s">
-        <v>45</v>
-      </c>
-      <c r="D3" s="84" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="77" t="s">
-        <v>64</v>
-      </c>
-      <c r="F3" s="54"/>
-      <c r="G3" s="78" t="s">
-        <v>86</v>
-      </c>
-      <c r="H3" s="78"/>
-    </row>
-    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="50"/>
-      <c r="B4" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="C4" s="65" t="s">
-        <v>45</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="72" t="s">
-        <v>65</v>
-      </c>
-      <c r="F4" s="55"/>
-      <c r="G4" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="H4" s="23"/>
-    </row>
-    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="50"/>
-      <c r="B5" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="C5" s="65" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" s="85" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="71" t="s">
-        <v>66</v>
-      </c>
-      <c r="F5" s="55"/>
-      <c r="G5" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="H5" s="23"/>
-    </row>
-    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="50">
-        <v>1</v>
-      </c>
-      <c r="B6" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" s="65" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="16" t="s">
+      <c r="F26" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G26" s="85" t="s">
+        <v>95</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="46"/>
+      <c r="B27" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="72" t="s">
-        <v>67</v>
-      </c>
-      <c r="F6" s="58" t="s">
-        <v>59</v>
-      </c>
-      <c r="G6" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="H6" s="23"/>
-    </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="50"/>
-      <c r="B7" s="26" t="s">
-        <v>73</v>
-      </c>
-      <c r="C7" s="65" t="s">
-        <v>45</v>
-      </c>
-      <c r="D7" s="85" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="71" t="s">
-        <v>68</v>
-      </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="H7" s="23"/>
-    </row>
-    <row r="8" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="50"/>
-      <c r="B8" s="82" t="s">
-        <v>74</v>
-      </c>
-      <c r="C8" s="81" t="s">
-        <v>45</v>
-      </c>
-      <c r="D8" s="79" t="s">
-        <v>75</v>
-      </c>
-      <c r="E8" s="83" t="s">
-        <v>69</v>
-      </c>
-      <c r="F8" s="56"/>
-      <c r="G8" s="80" t="s">
-        <v>86</v>
-      </c>
-      <c r="H8" s="80"/>
-    </row>
-    <row r="9" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="50"/>
-      <c r="B9" s="47" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="65" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="71" t="s">
-        <v>83</v>
-      </c>
-      <c r="E9" s="71" t="s">
-        <v>95</v>
-      </c>
-      <c r="F9" s="56"/>
-      <c r="G9" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="H9" s="23"/>
-    </row>
-    <row r="10" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="51"/>
-      <c r="B10" s="32"/>
-      <c r="C10" s="79"/>
-      <c r="D10" s="79"/>
-      <c r="E10" s="79"/>
-      <c r="F10" s="33"/>
-      <c r="G10" s="33"/>
-      <c r="H10" s="33"/>
-    </row>
-    <row r="11" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="49"/>
-      <c r="B11" s="42" t="s">
-        <v>54</v>
-      </c>
-      <c r="C11" s="64"/>
-      <c r="D11" s="86" t="s">
-        <v>87</v>
-      </c>
-      <c r="E11" s="86" t="s">
-        <v>88</v>
-      </c>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="44"/>
-    </row>
-    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="50"/>
-      <c r="B12" s="26" t="s">
-        <v>78</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="71" t="s">
-        <v>79</v>
-      </c>
-      <c r="E12" s="71" t="s">
-        <v>89</v>
-      </c>
-      <c r="F12" s="57"/>
-      <c r="G12" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="H12" s="23"/>
-    </row>
-    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="50"/>
-      <c r="B13" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" s="72" t="s">
-        <v>81</v>
-      </c>
-      <c r="E13" s="72" t="s">
-        <v>90</v>
-      </c>
-      <c r="F13" s="55"/>
-      <c r="G13" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="H13" s="23"/>
-    </row>
-    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="50"/>
-      <c r="B14" s="26" t="s">
-        <v>34</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" s="71" t="s">
-        <v>82</v>
-      </c>
-      <c r="E14" s="71" t="s">
-        <v>91</v>
-      </c>
-      <c r="F14" s="55"/>
-      <c r="G14" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="H14" s="23"/>
-    </row>
-    <row r="15" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="50">
-        <v>2</v>
-      </c>
-      <c r="B15" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="D15" s="72" t="s">
-        <v>84</v>
-      </c>
-      <c r="E15" s="72" t="s">
-        <v>92</v>
-      </c>
-      <c r="F15" s="58" t="s">
-        <v>60</v>
-      </c>
-      <c r="G15" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="H15" s="23"/>
-    </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="50"/>
-      <c r="B16" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="71" t="s">
-        <v>62</v>
-      </c>
-      <c r="E16" s="71" t="s">
-        <v>93</v>
-      </c>
-      <c r="F16" s="55"/>
-      <c r="G16" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="H16" s="23"/>
-    </row>
-    <row r="17" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="50"/>
-      <c r="B17" s="26" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="D17" s="72" t="s">
-        <v>85</v>
-      </c>
-      <c r="E17" s="72" t="s">
-        <v>94</v>
-      </c>
-      <c r="F17" s="55"/>
-      <c r="G17" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="H17" s="23"/>
-    </row>
-    <row r="18" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="51"/>
-      <c r="B18" s="32"/>
-      <c r="C18" s="66"/>
-      <c r="D18" s="66"/>
-      <c r="E18" s="66"/>
-      <c r="F18" s="59"/>
-      <c r="G18" s="38"/>
-      <c r="H18" s="38"/>
-    </row>
-    <row r="19" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="49"/>
-      <c r="B19" s="42" t="s">
+      <c r="E27" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="C19" s="64"/>
-      <c r="D19" s="64"/>
-      <c r="E19" s="64"/>
-      <c r="F19" s="53"/>
-      <c r="G19" s="43"/>
-      <c r="H19" s="44"/>
-    </row>
-    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="50"/>
-      <c r="B20" s="36" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" s="65" t="s">
-        <v>46</v>
-      </c>
-      <c r="D20" s="71" t="s">
-        <v>24</v>
-      </c>
-      <c r="E20" s="71" t="s">
-        <v>97</v>
-      </c>
-      <c r="F20" s="61"/>
-      <c r="G20" s="60" t="s">
-        <v>86</v>
-      </c>
-      <c r="H20" s="18"/>
-    </row>
-    <row r="21" spans="1:8" s="29" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="46">
-        <v>3</v>
-      </c>
-      <c r="B21" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="63" t="s">
-        <v>46</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F21" s="58" t="s">
-        <v>61</v>
-      </c>
-      <c r="G21" s="88" t="s">
-        <v>86</v>
-      </c>
-      <c r="H21" s="1"/>
-    </row>
-    <row r="22" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="50"/>
-      <c r="B22" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" s="63" t="s">
-        <v>46</v>
-      </c>
-      <c r="D22" s="87" t="s">
-        <v>25</v>
-      </c>
-      <c r="E22" s="87" t="s">
-        <v>99</v>
-      </c>
-      <c r="F22" s="62"/>
-      <c r="G22" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="51"/>
-      <c r="B23" s="35"/>
-      <c r="C23" s="67"/>
-      <c r="D23" s="67"/>
-      <c r="E23" s="67"/>
-      <c r="F23" s="38"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="34"/>
-    </row>
-    <row r="24" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="49"/>
-      <c r="B24" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="C24" s="64"/>
-      <c r="D24" s="64"/>
-      <c r="E24" s="64"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="44"/>
-    </row>
-    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="50"/>
-      <c r="B25" s="37" t="s">
-        <v>14</v>
-      </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="E25" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="F25" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="G25" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="H25" s="18"/>
-    </row>
-    <row r="26" spans="1:8" ht="75" x14ac:dyDescent="0.25">
-      <c r="A26" s="50">
-        <v>4</v>
-      </c>
-      <c r="B26" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="G26" s="89" t="s">
-        <v>103</v>
-      </c>
-      <c r="H26" s="10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="50"/>
-      <c r="B27" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="51"/>
-      <c r="B28" s="30"/>
-      <c r="C28" s="67"/>
-      <c r="D28" s="67"/>
-      <c r="E28" s="67"/>
-      <c r="F28" s="34"/>
-      <c r="G28" s="34"/>
-      <c r="H28" s="34"/>
+      <c r="A28" s="47"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="63"/>
+      <c r="D28" s="63"/>
+      <c r="E28" s="63"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="30"/>
     </row>
     <row r="29" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="52"/>
-      <c r="B29" s="42" t="s">
-        <v>52</v>
-      </c>
-      <c r="C29" s="64"/>
-      <c r="D29" s="64"/>
-      <c r="E29" s="64"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="43"/>
-      <c r="H29" s="44"/>
+      <c r="A29" s="48"/>
+      <c r="B29" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" s="60"/>
+      <c r="D29" s="60"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="40"/>
     </row>
     <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="50"/>
-      <c r="B30" s="31" t="s">
-        <v>18</v>
-      </c>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="E30" s="16"/>
-      <c r="F30" s="18"/>
-      <c r="G30" s="18"/>
-      <c r="H30" s="18"/>
+      <c r="A30" s="46"/>
+      <c r="B30" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E30" s="12"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
     </row>
     <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="50">
+      <c r="A31" s="46">
         <v>5</v>
       </c>
-      <c r="B31" s="27" t="s">
-        <v>15</v>
+      <c r="B31" s="23" t="s">
+        <v>7</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="2"/>
@@ -2616,194 +3002,44 @@
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="51"/>
+      <c r="A32" s="47"/>
       <c r="B32" s="4"/>
-      <c r="C32" s="67"/>
-      <c r="D32" s="67"/>
-      <c r="E32" s="67"/>
-      <c r="F32" s="34"/>
-      <c r="G32" s="34"/>
-      <c r="H32" s="34"/>
+      <c r="C32" s="63"/>
+      <c r="D32" s="63"/>
+      <c r="E32" s="63"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="30"/>
     </row>
     <row r="33" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="33"/>
-      <c r="B33" s="41"/>
-      <c r="C33" s="69"/>
-      <c r="D33" s="68"/>
-      <c r="E33" s="69"/>
-      <c r="F33" s="39"/>
-      <c r="G33" s="39"/>
-      <c r="H33" s="40"/>
+      <c r="A33" s="29"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="65"/>
+      <c r="D33" s="64"/>
+      <c r="E33" s="65"/>
+      <c r="F33" s="35"/>
+      <c r="G33" s="35"/>
+      <c r="H33" s="36"/>
     </row>
     <row r="34" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="35" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="48" t="s">
+      <c r="B35" s="44" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D36" s="25" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D36" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="E36" s="29" t="str">
+      <c r="E36" s="25" t="str">
         <f>LOWER(D36)</f>
         <v>&lt;&lt; matter.responsibleattorney.email &gt;&gt;</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C39" s="70"/>
-      <c r="D39" s="70"/>
-      <c r="E39" s="70"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1C990D1-0B88-44F6-819D-B6728E0DB287}">
-  <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="60.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="7"/>
-      <c r="B27" s="7"/>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="7"/>
-      <c r="B28" s="7"/>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="7"/>
-      <c r="B29" s="7"/>
-    </row>
-    <row r="30" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="8"/>
-      <c r="B30" s="8"/>
+      <c r="C39" s="66"/>
+      <c r="D39" s="66"/>
+      <c r="E39" s="66"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Issue with only being able to download the first 200 templates from the Clio Templates API Determined that the issue was due to the pagination token not being included in the request Updated iter_pages function to include the pagination token in the request
</commit_message>
<xml_diff>
--- a/Testing_Files/ClioCustomField_TestValidation.xlsx
+++ b/Testing_Files/ClioCustomField_TestValidation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/Testing_Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1353" documentId="8_{3120D6FD-25C6-47F0-8A39-89B25F99CA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DC883BE-39E7-4E39-8B61-BFE02F2D8F10}"/>
+  <xr:revisionPtr revIDLastSave="1370" documentId="8_{3120D6FD-25C6-47F0-8A39-89B25F99CA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D52F1F9F-37C5-4CC3-BAD7-30902E9907F1}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="46092" yWindow="12" windowWidth="23016" windowHeight="13656" activeTab="1" xr2:uid="{DF2C5E22-660C-4BCB-A765-9F1A84EF46AA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DF2C5E22-660C-4BCB-A765-9F1A84EF46AA}"/>
   </bookViews>
   <sheets>
     <sheet name="FuncTestingScenarios" sheetId="4" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="119">
   <si>
     <t>Fields that do not exist in lookup table</t>
   </si>
@@ -135,8 +135,274 @@
     <t>Notes</t>
   </si>
   <si>
-    <r>
-      <rPr>
+    <t>Templates</t>
+  </si>
+  <si>
+    <t>ExcelDocument_4NonDocxFile_UploadFolder.xlsx</t>
+  </si>
+  <si>
+    <t>Template_UpperLowerCaseTestingScenario.docx</t>
+  </si>
+  <si>
+    <t>TemplateTesting_MixedCase_Spacing_SplitLines_Scenarios.docx</t>
+  </si>
+  <si>
+    <t>TemplateTesting_TableHeaderFooter_Scenario.docx</t>
+  </si>
+  <si>
+    <t>ZeroByteBlankDoc_UploadFolder.docx</t>
+  </si>
+  <si>
+    <t>Expected Results</t>
+  </si>
+  <si>
+    <t>Actual Results</t>
+  </si>
+  <si>
+    <t>Fields Inside Tables / Headers / Footers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Templates with Abnormal Data Structures </t>
+  </si>
+  <si>
+    <t>Additional Testing Scenarios</t>
+  </si>
+  <si>
+    <t>Mixed Case / Spacing in Custom Fields - Postive Testing</t>
+  </si>
+  <si>
+    <t>Mixed Case / Spacing in Custom Fields - Negative Testing</t>
+  </si>
+  <si>
+    <t>Uppercase/Lower Case Testing Scenario does not follow the Positive/Negative Testing Basis</t>
+  </si>
+  <si>
+    <t>No Custom Field</t>
+  </si>
+  <si>
+    <t>Incorrect File Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zero Bytes File </t>
+  </si>
+  <si>
+    <t>Custom Fields are Updated Successfully with all the same spaces within the Custom Field Itself</t>
+  </si>
+  <si>
+    <t>Custom Fields are NOT Updated Successfully becaue the spaces within the CF within the Templates do not Match the CFs in Lookup Table</t>
+  </si>
+  <si>
+    <t>Custom Fields are Successfully Updated within each testing scenarios table, headers, and footers CF location</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.CaseNumber &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.ResponsibleAttorney_Change3SpaceEndCF   &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;   MATTER.CUSTOMFIELD.PLAINTIFFSNAMESHORT_Change3SpaceBegCF &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;   Matter.CustomField.PlaintiffsFullLegalName_Change3SpaceEndBegCF   &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CaseNumber_ChangeNoSpaceEndCF&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.DefendantsFullLegalName_ChangeNoSpaceBegCF &gt;&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;&lt;Matter.CustomField.Judge_ChangeNoSpaceEndBegCF&gt;&gt; </t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.Judge&gt;&gt;</t>
+  </si>
+  <si>
+    <t>Old Custom Fields in Templates</t>
+  </si>
+  <si>
+    <t>New Custom Fields in Lookup Tables</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Date.Verbose   &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;   Matter.CustomField.CaseNameLong &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;   Matter.CustomField.OcStreetAddress   &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.responsibleattorney.email &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.OcCityStateZip&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.CaseNameLong&gt;&gt;</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>Purposeply Slightly Incorrect CF Values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used to Validate Neg. Testing - If Below Values are Found Neg. Test Unsuccessfull </t>
+  </si>
+  <si>
+    <t>&lt;&lt; Date.Verbose_Change1&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;   Matter.CustomField.CaseNameLong_Change1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;   Matter.CustomField.OcStreetAddress_Change1   &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.OcCityStateZip_Change1&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.CaseNumber_Change1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.CaseNameLong_Change1&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.responsibleattorney.email_Change1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Success </t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.County_Change1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.OcCityStateZip_Change1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.OcStreetAddress_Change1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>Nothing Happens</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Script downloaded the Excel File as a .docx (unable to open) when running Script to Update for an Error --&gt; Need to edit script to either only download .docx files, because we created a corrupted file even if we tried to skip over Update Script trying to then skip over Upload Script is just too much hassel. Final conclusion need to restrict to only download .docx files. - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Completed Code Update to Skip Over Non - Word Docs</t>
+    </r>
+  </si>
+  <si>
+    <t>Skip Over Non-Word Document</t>
+  </si>
+  <si>
+    <t>After Code Change we now will skip over non-word template documents</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleYear &gt;&gt;</t>
+  </si>
+  <si>
+    <t>Old_Value</t>
+  </si>
+  <si>
+    <t>New_Value</t>
+  </si>
+  <si>
+    <t>&lt;&lt; date.verbose &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; date.verbose_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.casenumber &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.casenumber_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.county &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.county_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DefendantsNameShort &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DefendantsNameShort_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleYear_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CourtStreetAddress &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CourtStreetAddress_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;  TestCustomField.Test_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>CMS AB</t>
+  </si>
+  <si>
+    <t>CMS NonAB</t>
+  </si>
+  <si>
+    <t>NOD DLR 1</t>
+  </si>
+  <si>
+    <t>NOD DLR 2</t>
+  </si>
+  <si>
+    <t>SUBP No. 2</t>
+  </si>
+  <si>
+    <t>SUBP No. 3</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>TextBox</t>
+  </si>
+  <si>
+    <t>Shape</t>
+  </si>
+  <si>
+    <t>Body</t>
+  </si>
+  <si>
+    <t>Footers</t>
+  </si>
+  <si>
+    <t>Headers</t>
+  </si>
+  <si>
+    <t>Count of Custom Fields:</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Test.CustomField &gt;&gt;</t>
+  </si>
+  <si>
+    <t>Count of Updated Custom Fields:</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
         <i/>
         <sz val="11"/>
         <color theme="1"/>
@@ -148,18 +414,30 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>: 3 Spaces on End of CF (split between lines, 14 CFs Within Template)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3 Spaces on End of CF (split between lines, 14 CFs Within Template)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
         <i/>
         <sz val="11"/>
         <color theme="1"/>
@@ -167,7 +445,255 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">MCS Custom Field 3: </t>
+      <t>MCS Custom Field 2:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3 Spaces on Beginning of CF (split between pages,  6 Original CFs Within Template, 1 Test CF)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 3:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3 Spaces on Both Beg. and End of CF (2 Original CFs Within Template, 1 Test CF)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 4:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>No Spaces on End of CF (2 Original CFs Within Template. 1 Test CF)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 5:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> No Spaces on Beg. of CF (2 Original CFs Within Template. 1 Test CF)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 6:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>No Spaces on Both Beg. And End of CF (2 Original CFs Within Template. 1 Test CF)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 7:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> CF in Uppercase in Template, While Lowercase in Lookuptable</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 1</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 3 Spaces on End of CF </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 2:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 3 Spaces on Beginning of CF </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 3:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
@@ -183,6 +709,7 @@
   <si>
     <r>
       <rPr>
+        <b/>
         <i/>
         <sz val="11"/>
         <color theme="1"/>
@@ -206,6 +733,7 @@
   <si>
     <r>
       <rPr>
+        <b/>
         <i/>
         <sz val="11"/>
         <color theme="1"/>
@@ -217,18 +745,30 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> No Spaces on Beg. of CF (3 CFs Within Template)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>No Spaces on Beg. of CF (3 CFs Within Template)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
         <i/>
         <sz val="11"/>
         <color theme="1"/>
@@ -240,18 +780,30 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> No Spaces on Both Beg. And End of CF (3 CFs Within Template)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>No Spaces on Both Beg. And End of CF (3 CFs Within Template)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
         <i/>
         <sz val="11"/>
         <color theme="1"/>
@@ -263,18 +815,30 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Tables (CF in Table, But Also in Paragraph) </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Tables (CF in Table, But Also in Paragraph) </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
         <i/>
         <sz val="11"/>
         <color theme="1"/>
@@ -286,18 +850,30 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Headers (CF in Header, But Also in Paragraph) </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Headers (CF in Header, But Also in Paragraph) </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
         <i/>
         <sz val="11"/>
         <color theme="1"/>
@@ -305,7 +881,18 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Inside THF Custom Field 3: </t>
+      <t>Inside THF Custom Field 3:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
@@ -317,430 +904,6 @@
       </rPr>
       <t>Footers (CF Only in Footer)</t>
     </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>MCS Custom Field 7:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> CF in Uppercase in Template, While Lowercase in Lookuptable</t>
-    </r>
-  </si>
-  <si>
-    <t>Templates</t>
-  </si>
-  <si>
-    <t>ExcelDocument_4NonDocxFile_UploadFolder.xlsx</t>
-  </si>
-  <si>
-    <t>Template_UpperLowerCaseTestingScenario.docx</t>
-  </si>
-  <si>
-    <t>TemplateTesting_MixedCase_Spacing_SplitLines_Scenarios.docx</t>
-  </si>
-  <si>
-    <t>TemplateTesting_TableHeaderFooter_Scenario.docx</t>
-  </si>
-  <si>
-    <t>ZeroByteBlankDoc_UploadFolder.docx</t>
-  </si>
-  <si>
-    <t>Expected Results</t>
-  </si>
-  <si>
-    <t>Actual Results</t>
-  </si>
-  <si>
-    <t>Fields Inside Tables / Headers / Footers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Templates with Abnormal Data Structures </t>
-  </si>
-  <si>
-    <t>Additional Testing Scenarios</t>
-  </si>
-  <si>
-    <t>Mixed Case / Spacing in Custom Fields - Postive Testing</t>
-  </si>
-  <si>
-    <t>Mixed Case / Spacing in Custom Fields - Negative Testing</t>
-  </si>
-  <si>
-    <t>Uppercase/Lower Case Testing Scenario does not follow the Positive/Negative Testing Basis</t>
-  </si>
-  <si>
-    <t>No Custom Field</t>
-  </si>
-  <si>
-    <t>Incorrect File Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zero Bytes File </t>
-  </si>
-  <si>
-    <t>Custom Fields are Updated Successfully with all the same spaces within the Custom Field Itself</t>
-  </si>
-  <si>
-    <t>Custom Fields are NOT Updated Successfully becaue the spaces within the CF within the Templates do not Match the CFs in Lookup Table</t>
-  </si>
-  <si>
-    <t>Custom Fields are Successfully Updated within each testing scenarios table, headers, and footers CF location</t>
-  </si>
-  <si>
-    <t>&lt;&lt;Matter.CustomField.CaseNumber &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; MATTER.RESPONSIBLEATTORNEY.EMAIL &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.ResponsibleAttorney_Change3SpaceEndCF   &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;   MATTER.CUSTOMFIELD.PLAINTIFFSNAMESHORT_Change3SpaceBegCF &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;   Matter.CustomField.PlaintiffsFullLegalName_Change3SpaceEndBegCF   &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.CaseNumber_ChangeNoSpaceEndCF&gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;Matter.CustomField.DefendantsFullLegalName_ChangeNoSpaceBegCF &gt;&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;&lt;Matter.CustomField.Judge_ChangeNoSpaceEndBegCF&gt;&gt; </t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">MCS Custom Field 2: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>3 Spaces on Beginning of CF (split between pages,  6 Original CFs Within Template, 1 Test CF)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">MCS Custom Field 3: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>3 Spaces on Both Beg. and End of CF (2 Original CFs Within Template, 1 Test CF)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>MCS Custom Field 4:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>No Spaces on End of CF (2 Original CFs Within Template. 1 Test CF)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>MCS Custom Field 5:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> No Spaces on Beg. of CF (2 Original CFs Within Template. 1 Test CF)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>MCS Custom Field 6:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> No Spaces on Both Beg. And End of CF (2 Original CFs Within Template. 1 Test CF)</t>
-    </r>
-  </si>
-  <si>
-    <t>&lt;&lt;Matter.CustomField.Judge&gt;&gt;</t>
-  </si>
-  <si>
-    <t>Old Custom Fields in Templates</t>
-  </si>
-  <si>
-    <t>New Custom Fields in Lookup Tables</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>MCS Custom Field 1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">: 3 Spaces on End of CF </t>
-    </r>
-  </si>
-  <si>
-    <t>&lt;&lt; Date.Verbose   &gt;&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCS Custom Field 2: 3 Spaces on Beginning of CF </t>
-  </si>
-  <si>
-    <t>&lt;&lt;   Matter.CustomField.CaseNameLong &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;   Matter.CustomField.OcStreetAddress   &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.responsibleattorney.email &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.OcCityStateZip&gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;Matter.CustomField.CaseNameLong&gt;&gt;</t>
-  </si>
-  <si>
-    <t>Success</t>
-  </si>
-  <si>
-    <t>Purposeply Slightly Incorrect CF Values</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Used to Validate Neg. Testing - If Below Values are Found Neg. Test Unsuccessfull </t>
-  </si>
-  <si>
-    <t>&lt;&lt; Date.Verbose_Change1&gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;   Matter.CustomField.CaseNameLong_Change1 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;   Matter.CustomField.OcStreetAddress_Change1   &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.OcCityStateZip_Change1&gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;Matter.CustomField.CaseNumber_Change1 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;Matter.CustomField.CaseNameLong_Change1&gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.responsibleattorney.email_Change1 &gt;&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Success </t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.County_Change1 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.OcCityStateZip_Change1 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.OcStreetAddress_Change1 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>Nothing Happens</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Script downloaded the Excel File as a .docx (unable to open) when running Script to Update for an Error --&gt; Need to edit script to either only download .docx files, because we created a corrupted file even if we tried to skip over Update Script trying to then skip over Upload Script is just too much hassel. Final conclusion need to restrict to only download .docx files. - </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Completed Code Update to Skip Over Non - Word Docs</t>
-    </r>
-  </si>
-  <si>
-    <t>Skip Over Non-Word Document</t>
-  </si>
-  <si>
-    <t>After Code Change we now will skip over non-word template documents</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.VehicleYear &gt;&gt;</t>
-  </si>
-  <si>
-    <t>Old_Value</t>
-  </si>
-  <si>
-    <t>New_Value</t>
-  </si>
-  <si>
-    <t>&lt;&lt; date.verbose &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; date.verbose_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.casenumber &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.casenumber_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.county &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.county_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.DefendantsNameShort &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.DefendantsNameShort_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.VehicleYear_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.CourtStreetAddress &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.CourtStreetAddress_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;  TestCustomField.Test_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>CMS AB</t>
-  </si>
-  <si>
-    <t>CMS NonAB</t>
-  </si>
-  <si>
-    <t>NOD DLR 1</t>
-  </si>
-  <si>
-    <t>NOD DLR 2</t>
-  </si>
-  <si>
-    <t>SUBP No. 2</t>
-  </si>
-  <si>
-    <t>SUBP No. 3</t>
-  </si>
-  <si>
-    <t>Location</t>
-  </si>
-  <si>
-    <t>TextBox</t>
-  </si>
-  <si>
-    <t>Shape</t>
-  </si>
-  <si>
-    <t>Body</t>
-  </si>
-  <si>
-    <t>Footers</t>
-  </si>
-  <si>
-    <t>Headers</t>
-  </si>
-  <si>
-    <t>Count of Custom Fields:</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Test.CustomField &gt;&gt;</t>
-  </si>
-  <si>
-    <t>Count of Updated Custom Fields:</t>
   </si>
 </sst>
 </file>
@@ -2285,30 +2448,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="76" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="76" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1" s="76" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" s="76" t="s">
+        <v>90</v>
+      </c>
+      <c r="E1" s="76" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="76" t="s">
-        <v>105</v>
-      </c>
-      <c r="C1" s="76" t="s">
-        <v>106</v>
-      </c>
-      <c r="D1" s="76" t="s">
-        <v>107</v>
-      </c>
-      <c r="E1" s="76" t="s">
-        <v>108</v>
-      </c>
       <c r="F1" s="76" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
       <c r="G1" s="76" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="78" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="B2" s="87">
         <v>4</v>
@@ -2331,7 +2494,7 @@
     </row>
     <row r="3" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="79" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="B3" s="80"/>
       <c r="C3" s="81"/>
@@ -2342,7 +2505,7 @@
     </row>
     <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="B4" s="7">
         <v>2</v>
@@ -2361,7 +2524,7 @@
     </row>
     <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -2372,7 +2535,7 @@
     </row>
     <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="B6" s="1">
         <v>2</v>
@@ -2391,7 +2554,7 @@
     </row>
     <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -2402,7 +2565,7 @@
     </row>
     <row r="8" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="20" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="B8" s="53"/>
       <c r="C8" s="53"/>
@@ -2422,7 +2585,7 @@
     </row>
     <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="83" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="B10" s="88">
         <v>6</v>
@@ -2445,7 +2608,7 @@
     </row>
     <row r="11" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="77" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="B11" s="80"/>
       <c r="C11" s="81"/>
@@ -2456,7 +2619,7 @@
     </row>
     <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="B12" s="7">
         <v>6</v>
@@ -2475,7 +2638,7 @@
     </row>
     <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -2486,7 +2649,7 @@
     </row>
     <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -2501,7 +2664,7 @@
     </row>
     <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -2512,7 +2675,7 @@
     </row>
     <row r="16" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="20" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="B16" s="53"/>
       <c r="C16" s="53"/>
@@ -2532,7 +2695,7 @@
     </row>
     <row r="18" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="78" t="s">
-        <v>97</v>
+        <v>80</v>
       </c>
       <c r="B18" s="87">
         <v>2</v>
@@ -2555,7 +2718,7 @@
     </row>
     <row r="19" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="77" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="B19" s="80"/>
       <c r="C19" s="81"/>
@@ -2566,7 +2729,7 @@
     </row>
     <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="B20" s="7">
         <v>2</v>
@@ -2585,7 +2748,7 @@
     </row>
     <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -2596,7 +2759,7 @@
     </row>
     <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -2611,7 +2774,7 @@
     </row>
     <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -2622,7 +2785,7 @@
     </row>
     <row r="24" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="20" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="B24" s="53"/>
       <c r="C24" s="53"/>
@@ -2642,7 +2805,7 @@
     </row>
     <row r="26" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="78" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="B26" s="87">
         <v>6</v>
@@ -2665,7 +2828,7 @@
     </row>
     <row r="27" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="77" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="B27" s="80"/>
       <c r="C27" s="81"/>
@@ -2676,7 +2839,7 @@
     </row>
     <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="B28" s="7">
         <v>6</v>
@@ -2695,7 +2858,7 @@
     </row>
     <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2706,7 +2869,7 @@
     </row>
     <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -2717,7 +2880,7 @@
     </row>
     <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -2728,7 +2891,7 @@
     </row>
     <row r="32" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -2748,7 +2911,7 @@
     </row>
     <row r="34" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="78" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="B34" s="87">
         <v>0</v>
@@ -2771,7 +2934,7 @@
     </row>
     <row r="35" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="77" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="B35" s="80"/>
       <c r="C35" s="81"/>
@@ -2782,7 +2945,7 @@
     </row>
     <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
@@ -2793,7 +2956,7 @@
     </row>
     <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -2804,7 +2967,7 @@
     </row>
     <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -2819,7 +2982,7 @@
     </row>
     <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -2830,7 +2993,7 @@
     </row>
     <row r="40" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -2850,7 +3013,7 @@
     </row>
     <row r="42" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="78" t="s">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="B42" s="87">
         <v>4</v>
@@ -2873,7 +3036,7 @@
     </row>
     <row r="43" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="77" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="B43" s="80"/>
       <c r="C43" s="81"/>
@@ -2884,7 +3047,7 @@
     </row>
     <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="B44" s="7">
         <v>4</v>
@@ -2903,7 +3066,7 @@
     </row>
     <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -2914,7 +3077,7 @@
     </row>
     <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -2925,7 +3088,7 @@
     </row>
     <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -2936,7 +3099,7 @@
     </row>
     <row r="48" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="20" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="B48" s="53"/>
       <c r="C48" s="53"/>
@@ -2956,7 +3119,7 @@
     </row>
     <row r="50" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="78" t="s">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="B50" s="87"/>
       <c r="C50" s="87"/>
@@ -2971,7 +3134,7 @@
     </row>
     <row r="51" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="77" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="B51" s="80"/>
       <c r="C51" s="81"/>
@@ -2982,7 +3145,7 @@
     </row>
     <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="7"/>
@@ -2997,7 +3160,7 @@
     </row>
     <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -3008,7 +3171,7 @@
     </row>
     <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -3019,7 +3182,7 @@
     </row>
     <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -3030,7 +3193,7 @@
     </row>
     <row r="56" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="20" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="B56" s="53"/>
       <c r="C56" s="53"/>
@@ -3050,7 +3213,7 @@
     </row>
     <row r="58" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="85" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="B58" s="86">
         <f>SUM(B50,B42,B34,B26,B18,B10,B2)</f>
@@ -3079,30 +3242,30 @@
     </row>
     <row r="61" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="91" t="s">
+        <v>75</v>
+      </c>
+      <c r="B61" s="92" t="s">
+        <v>88</v>
+      </c>
+      <c r="C61" s="92" t="s">
+        <v>89</v>
+      </c>
+      <c r="D61" s="92" t="s">
+        <v>90</v>
+      </c>
+      <c r="E61" s="92" t="s">
+        <v>91</v>
+      </c>
+      <c r="F61" s="92" t="s">
         <v>92</v>
       </c>
-      <c r="B61" s="92" t="s">
-        <v>105</v>
-      </c>
-      <c r="C61" s="92" t="s">
-        <v>106</v>
-      </c>
-      <c r="D61" s="92" t="s">
-        <v>107</v>
-      </c>
-      <c r="E61" s="92" t="s">
-        <v>108</v>
-      </c>
-      <c r="F61" s="92" t="s">
-        <v>109</v>
-      </c>
       <c r="G61" s="93" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="96" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="B62" s="99">
         <v>4</v>
@@ -3134,7 +3297,7 @@
     </row>
     <row r="64" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="96" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="B64" s="99">
         <v>6</v>
@@ -3166,7 +3329,7 @@
     </row>
     <row r="66" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="96" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="B66" s="99">
         <v>2</v>
@@ -3198,7 +3361,7 @@
     </row>
     <row r="68" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="96" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="B68" s="99">
         <v>6</v>
@@ -3230,7 +3393,7 @@
     </row>
     <row r="70" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="96" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="B70" s="99">
         <v>0</v>
@@ -3262,7 +3425,7 @@
     </row>
     <row r="72" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="96" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="B72" s="99">
         <v>4</v>
@@ -3294,7 +3457,7 @@
     </row>
     <row r="74" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="96" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="B74" s="99">
         <v>0</v>
@@ -3326,7 +3489,7 @@
     </row>
     <row r="76" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="98" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="B76" s="108">
         <f>SUM(B62:B75)</f>
@@ -3383,19 +3546,19 @@
         <v>13</v>
       </c>
       <c r="C1" s="60" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="D1" s="60" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="E1" s="60" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="F1" s="60" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="G1" s="60" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="H1" s="60" t="s">
         <v>18</v>
@@ -3404,7 +3567,7 @@
     <row r="2" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="35"/>
       <c r="B2" s="28" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C2" s="50"/>
       <c r="D2" s="50"/>
@@ -3413,63 +3576,63 @@
       <c r="G2" s="29"/>
       <c r="H2" s="30"/>
     </row>
-    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="36"/>
       <c r="B3" s="61" t="s">
-        <v>19</v>
+        <v>103</v>
       </c>
       <c r="C3" s="62" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D3" s="70" t="s">
         <v>7</v>
       </c>
       <c r="E3" s="63" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F3" s="40"/>
       <c r="G3" s="64" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H3" s="64"/>
     </row>
     <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="36"/>
       <c r="B4" s="14" t="s">
-        <v>56</v>
+        <v>104</v>
       </c>
       <c r="C4" s="51" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>5</v>
       </c>
       <c r="E4" s="58" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="F4" s="41"/>
       <c r="G4" s="9" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H4" s="9"/>
     </row>
     <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="36"/>
       <c r="B5" s="12" t="s">
-        <v>57</v>
+        <v>105</v>
       </c>
       <c r="C5" s="51" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D5" s="71" t="s">
         <v>6</v>
       </c>
       <c r="E5" s="57" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="F5" s="41"/>
       <c r="G5" s="9" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H5" s="9"/>
     </row>
@@ -3478,82 +3641,82 @@
         <v>1</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>58</v>
+        <v>106</v>
       </c>
       <c r="C6" s="51" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>8</v>
       </c>
       <c r="E6" s="58" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F6" s="44" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H6" s="9"/>
     </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="36"/>
       <c r="B7" s="12" t="s">
-        <v>59</v>
+        <v>107</v>
       </c>
       <c r="C7" s="51" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D7" s="71" t="s">
         <v>9</v>
       </c>
       <c r="E7" s="57" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="F7" s="41"/>
       <c r="G7" s="9" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H7" s="9"/>
     </row>
     <row r="8" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="36"/>
       <c r="B8" s="68" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
       <c r="C8" s="67" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D8" s="65" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="E8" s="69" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="F8" s="42"/>
       <c r="G8" s="66" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H8" s="66"/>
     </row>
-    <row r="9" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="36"/>
       <c r="B9" s="33" t="s">
-        <v>27</v>
+        <v>109</v>
       </c>
       <c r="C9" s="51" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="D9" s="57" t="s">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="E9" s="57" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="F9" s="42"/>
       <c r="G9" s="9" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="H9" s="9"/>
     </row>
@@ -3570,14 +3733,14 @@
     <row r="11" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="35"/>
       <c r="B11" s="28" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C11" s="50"/>
       <c r="D11" s="72" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="E11" s="72" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="F11" s="29"/>
       <c r="G11" s="29"/>
@@ -3586,60 +3749,60 @@
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="36"/>
       <c r="B12" s="12" t="s">
-        <v>64</v>
+        <v>110</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D12" s="57" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="E12" s="57" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="F12" s="43"/>
       <c r="G12" s="9" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="H12" s="9"/>
     </row>
     <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="36"/>
       <c r="B13" s="14" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D13" s="58" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="E13" s="58" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="F13" s="41"/>
       <c r="G13" s="9" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="H13" s="9"/>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="36"/>
       <c r="B14" s="12" t="s">
-        <v>20</v>
+        <v>112</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D14" s="57" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="E14" s="57" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F14" s="41"/>
       <c r="G14" s="9" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="H14" s="9"/>
     </row>
@@ -3648,62 +3811,62 @@
         <v>2</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>21</v>
+        <v>113</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D15" s="58" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="E15" s="58" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="F15" s="44" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="H15" s="9"/>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="36"/>
       <c r="B16" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>31</v>
-      </c>
       <c r="D16" s="57" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E16" s="57" t="s">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="F16" s="41"/>
       <c r="G16" s="9" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="H16" s="9"/>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="36"/>
       <c r="B17" s="12" t="s">
-        <v>23</v>
+        <v>115</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D17" s="58" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="E17" s="58" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="F17" s="41"/>
       <c r="G17" s="9" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="H17" s="9"/>
     </row>
@@ -3720,7 +3883,7 @@
     <row r="19" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="35"/>
       <c r="B19" s="28" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="C19" s="50"/>
       <c r="D19" s="50"/>
@@ -3732,20 +3895,20 @@
     <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="36"/>
       <c r="B20" s="22" t="s">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="C20" s="51" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D20" s="57" t="s">
         <v>10</v>
       </c>
       <c r="E20" s="57" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="F20" s="47"/>
       <c r="G20" s="46" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H20" s="8"/>
     </row>
@@ -3754,42 +3917,42 @@
         <v>3</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>25</v>
+        <v>117</v>
       </c>
       <c r="C21" s="49" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="F21" s="44" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="G21" s="74" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H21" s="1"/>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="36"/>
       <c r="B22" s="11" t="s">
-        <v>26</v>
+        <v>118</v>
       </c>
       <c r="C22" s="49" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D22" s="73" t="s">
         <v>11</v>
       </c>
       <c r="E22" s="73" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="F22" s="48"/>
       <c r="G22" s="6" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H22" s="2"/>
     </row>
@@ -3806,7 +3969,7 @@
     <row r="24" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="35"/>
       <c r="B24" s="28" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C24" s="50"/>
       <c r="D24" s="50"/>
@@ -3825,13 +3988,13 @@
         <v>14</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H25" s="8"/>
     </row>
@@ -3843,22 +4006,22 @@
         <v>2</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>15</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="G26" s="75" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3867,13 +4030,13 @@
         <v>3</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>16</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -3892,7 +4055,7 @@
     <row r="29" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="38"/>
       <c r="B29" s="28" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="C29" s="50"/>
       <c r="D29" s="50"/>
@@ -3954,16 +4117,7 @@
     <row r="34" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="35" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="34" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D36" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="E36" s="15" t="str">
-        <f>LOWER(D36)</f>
-        <v>&lt;&lt; matter.responsibleattorney.email &gt;&gt;</v>
+        <v>32</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">

</xml_diff>